<commit_message>
coordinates sent to nabin sir and others minor edits
</commit_message>
<xml_diff>
--- a/ward 1 yojana haru.xlsx
+++ b/ward 1 yojana haru.xlsx
@@ -1,23 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29029"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="G:\2082_2083\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E83202CE-0298-4777-A431-2BF54AC76631}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B7BAE08A-802D-4D52-8C91-6DE223898FFC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="nagar stariya" sheetId="1" r:id="rId1"/>
+    <sheet name="nagar stariya (2)" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Area" localSheetId="0">'nagar stariya'!$B$6:$E$59</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="1">'nagar stariya (2)'!$B$6:$E$59</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'nagar stariya'!$6:$6</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="1">'nagar stariya (2)'!$6:$6</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -38,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="186" uniqueCount="124">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="372" uniqueCount="124">
   <si>
     <t>qm= ;+=</t>
   </si>
@@ -416,7 +419,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -451,6 +454,11 @@
     <font>
       <b/>
       <sz val="14"/>
+      <color theme="1"/>
+      <name val="Preeti"/>
+    </font>
+    <font>
+      <sz val="16"/>
       <color theme="1"/>
       <name val="Preeti"/>
     </font>
@@ -490,7 +498,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -534,6 +542,30 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="6" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1758,4 +1790,951 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" scale="80" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F4E01FAB-A237-4A57-9FE8-1F71349717D9}">
+  <dimension ref="B1:H63"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="8" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="65.7109375" customWidth="1"/>
+    <col min="4" max="4" width="19.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="15.140625" customWidth="1"/>
+    <col min="6" max="6" width="11.140625" customWidth="1"/>
+    <col min="7" max="7" width="13.42578125" customWidth="1"/>
+    <col min="8" max="8" width="10.5703125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="2:8" ht="19.5" x14ac:dyDescent="0.25">
+      <c r="B1" s="17" t="s">
+        <v>7</v>
+      </c>
+      <c r="C1" s="17"/>
+      <c r="D1" s="17"/>
+      <c r="E1" s="17"/>
+      <c r="F1" s="17"/>
+      <c r="G1" s="17"/>
+      <c r="H1" s="17"/>
+    </row>
+    <row r="2" spans="2:8" ht="19.5" x14ac:dyDescent="0.25">
+      <c r="B2" s="17" t="s">
+        <v>8</v>
+      </c>
+      <c r="C2" s="17"/>
+      <c r="D2" s="17"/>
+      <c r="E2" s="17"/>
+      <c r="F2" s="17"/>
+      <c r="G2" s="17"/>
+      <c r="H2" s="17"/>
+    </row>
+    <row r="3" spans="2:8" ht="19.5" x14ac:dyDescent="0.25">
+      <c r="B3" s="17" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3" s="17"/>
+      <c r="D3" s="17"/>
+      <c r="E3" s="17"/>
+      <c r="F3" s="17"/>
+      <c r="G3" s="17"/>
+      <c r="H3" s="17"/>
+    </row>
+    <row r="4" spans="2:8" ht="19.5" x14ac:dyDescent="0.25">
+      <c r="B4" s="2"/>
+      <c r="C4" s="2"/>
+      <c r="D4" s="2"/>
+      <c r="E4" s="2"/>
+      <c r="F4" s="2"/>
+      <c r="G4" s="2"/>
+      <c r="H4" s="5" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="5" spans="2:8" ht="21" x14ac:dyDescent="0.35">
+      <c r="B5" s="3"/>
+      <c r="C5" s="3"/>
+      <c r="D5" s="3"/>
+      <c r="E5" s="3"/>
+      <c r="F5" s="3"/>
+      <c r="G5" s="3"/>
+      <c r="H5" s="3"/>
+    </row>
+    <row r="6" spans="2:8" s="1" customFormat="1" ht="19.5" x14ac:dyDescent="0.25">
+      <c r="B6" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="C6" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="D6" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="E6" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="F6" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="G6" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="H6" s="4" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="7" spans="2:8" s="1" customFormat="1" ht="19.5" x14ac:dyDescent="0.25">
+      <c r="B7" s="4"/>
+      <c r="C7" s="18" t="s">
+        <v>39</v>
+      </c>
+      <c r="D7" s="4"/>
+      <c r="E7" s="4"/>
+      <c r="F7" s="4"/>
+      <c r="G7" s="4"/>
+      <c r="H7" s="4"/>
+    </row>
+    <row r="8" spans="2:8" s="12" customFormat="1" ht="19.5" x14ac:dyDescent="0.25">
+      <c r="B8" s="19" t="s">
+        <v>14</v>
+      </c>
+      <c r="C8" s="20" t="s">
+        <v>11</v>
+      </c>
+      <c r="D8" s="20" t="s">
+        <v>12</v>
+      </c>
+      <c r="E8" s="20" t="s">
+        <v>13</v>
+      </c>
+      <c r="F8" s="9"/>
+      <c r="G8" s="9"/>
+      <c r="H8" s="9"/>
+    </row>
+    <row r="9" spans="2:8" s="12" customFormat="1" ht="19.5" x14ac:dyDescent="0.25">
+      <c r="B9" s="19" t="s">
+        <v>15</v>
+      </c>
+      <c r="C9" s="20" t="s">
+        <v>123</v>
+      </c>
+      <c r="D9" s="20" t="s">
+        <v>12</v>
+      </c>
+      <c r="E9" s="20" t="s">
+        <v>13</v>
+      </c>
+      <c r="F9" s="9"/>
+      <c r="G9" s="9"/>
+      <c r="H9" s="9"/>
+    </row>
+    <row r="10" spans="2:8" s="12" customFormat="1" ht="19.5" x14ac:dyDescent="0.25">
+      <c r="B10" s="20" t="s">
+        <v>26</v>
+      </c>
+      <c r="C10" s="20" t="s">
+        <v>16</v>
+      </c>
+      <c r="D10" s="20" t="s">
+        <v>12</v>
+      </c>
+      <c r="E10" s="20" t="s">
+        <v>13</v>
+      </c>
+      <c r="F10" s="9"/>
+      <c r="G10" s="9"/>
+      <c r="H10" s="9"/>
+    </row>
+    <row r="11" spans="2:8" s="12" customFormat="1" ht="19.5" x14ac:dyDescent="0.25">
+      <c r="B11" s="20" t="s">
+        <v>27</v>
+      </c>
+      <c r="C11" s="20" t="s">
+        <v>17</v>
+      </c>
+      <c r="D11" s="20" t="s">
+        <v>12</v>
+      </c>
+      <c r="E11" s="20" t="s">
+        <v>18</v>
+      </c>
+      <c r="F11" s="9"/>
+      <c r="G11" s="9"/>
+      <c r="H11" s="9"/>
+    </row>
+    <row r="12" spans="2:8" s="12" customFormat="1" ht="19.5" x14ac:dyDescent="0.25">
+      <c r="B12" s="20" t="s">
+        <v>28</v>
+      </c>
+      <c r="C12" s="20" t="s">
+        <v>19</v>
+      </c>
+      <c r="D12" s="20" t="s">
+        <v>12</v>
+      </c>
+      <c r="E12" s="20" t="s">
+        <v>20</v>
+      </c>
+      <c r="F12" s="9"/>
+      <c r="G12" s="9"/>
+      <c r="H12" s="9"/>
+    </row>
+    <row r="13" spans="2:8" s="12" customFormat="1" ht="19.5" x14ac:dyDescent="0.25">
+      <c r="B13" s="20" t="s">
+        <v>29</v>
+      </c>
+      <c r="C13" s="20" t="s">
+        <v>21</v>
+      </c>
+      <c r="D13" s="20" t="s">
+        <v>12</v>
+      </c>
+      <c r="E13" s="20" t="s">
+        <v>18</v>
+      </c>
+      <c r="F13" s="9"/>
+      <c r="G13" s="9"/>
+      <c r="H13" s="9"/>
+    </row>
+    <row r="14" spans="2:8" s="12" customFormat="1" ht="78" x14ac:dyDescent="0.25">
+      <c r="B14" s="20" t="s">
+        <v>30</v>
+      </c>
+      <c r="C14" s="21" t="s">
+        <v>22</v>
+      </c>
+      <c r="D14" s="20" t="s">
+        <v>12</v>
+      </c>
+      <c r="E14" s="20" t="s">
+        <v>23</v>
+      </c>
+      <c r="F14" s="9"/>
+      <c r="G14" s="9"/>
+      <c r="H14" s="9"/>
+    </row>
+    <row r="15" spans="2:8" s="12" customFormat="1" ht="19.5" x14ac:dyDescent="0.25">
+      <c r="B15" s="20" t="s">
+        <v>31</v>
+      </c>
+      <c r="C15" s="21" t="s">
+        <v>24</v>
+      </c>
+      <c r="D15" s="20" t="s">
+        <v>12</v>
+      </c>
+      <c r="E15" s="20" t="s">
+        <v>13</v>
+      </c>
+      <c r="F15" s="9"/>
+      <c r="G15" s="9"/>
+      <c r="H15" s="9"/>
+    </row>
+    <row r="16" spans="2:8" s="12" customFormat="1" ht="19.5" x14ac:dyDescent="0.25">
+      <c r="B16" s="20" t="s">
+        <v>32</v>
+      </c>
+      <c r="C16" s="21" t="s">
+        <v>25</v>
+      </c>
+      <c r="D16" s="20" t="s">
+        <v>12</v>
+      </c>
+      <c r="E16" s="20" t="s">
+        <v>23</v>
+      </c>
+      <c r="F16" s="9"/>
+      <c r="G16" s="9"/>
+      <c r="H16" s="9"/>
+    </row>
+    <row r="17" spans="2:8" s="12" customFormat="1" ht="19.5" x14ac:dyDescent="0.25">
+      <c r="B17" s="20"/>
+      <c r="C17" s="22" t="s">
+        <v>38</v>
+      </c>
+      <c r="D17" s="20"/>
+      <c r="E17" s="20"/>
+      <c r="F17" s="9"/>
+      <c r="G17" s="9"/>
+      <c r="H17" s="9"/>
+    </row>
+    <row r="18" spans="2:8" s="12" customFormat="1" ht="97.5" x14ac:dyDescent="0.25">
+      <c r="B18" s="20" t="s">
+        <v>66</v>
+      </c>
+      <c r="C18" s="21" t="s">
+        <v>33</v>
+      </c>
+      <c r="D18" s="23" t="s">
+        <v>35</v>
+      </c>
+      <c r="E18" s="24" t="s">
+        <v>34</v>
+      </c>
+      <c r="F18" s="9"/>
+      <c r="G18" s="9"/>
+      <c r="H18" s="9"/>
+    </row>
+    <row r="19" spans="2:8" s="12" customFormat="1" ht="39" x14ac:dyDescent="0.25">
+      <c r="B19" s="20" t="s">
+        <v>67</v>
+      </c>
+      <c r="C19" s="21" t="s">
+        <v>36</v>
+      </c>
+      <c r="D19" s="23" t="s">
+        <v>35</v>
+      </c>
+      <c r="E19" s="20" t="s">
+        <v>23</v>
+      </c>
+      <c r="F19" s="9"/>
+      <c r="G19" s="9"/>
+      <c r="H19" s="9"/>
+    </row>
+    <row r="20" spans="2:8" s="12" customFormat="1" ht="39" x14ac:dyDescent="0.25">
+      <c r="B20" s="20" t="s">
+        <v>121</v>
+      </c>
+      <c r="C20" s="20" t="s">
+        <v>122</v>
+      </c>
+      <c r="D20" s="23" t="s">
+        <v>35</v>
+      </c>
+      <c r="E20" s="20" t="s">
+        <v>37</v>
+      </c>
+      <c r="F20" s="9"/>
+      <c r="G20" s="9"/>
+      <c r="H20" s="9"/>
+    </row>
+    <row r="21" spans="2:8" s="12" customFormat="1" ht="19.5" x14ac:dyDescent="0.25">
+      <c r="B21" s="20"/>
+      <c r="C21" s="25" t="s">
+        <v>40</v>
+      </c>
+      <c r="D21" s="20"/>
+      <c r="E21" s="20"/>
+      <c r="F21" s="9"/>
+      <c r="G21" s="9"/>
+      <c r="H21" s="9"/>
+    </row>
+    <row r="22" spans="2:8" s="12" customFormat="1" ht="58.5" x14ac:dyDescent="0.25">
+      <c r="B22" s="20" t="s">
+        <v>68</v>
+      </c>
+      <c r="C22" s="20" t="s">
+        <v>42</v>
+      </c>
+      <c r="D22" s="21" t="s">
+        <v>41</v>
+      </c>
+      <c r="E22" s="20" t="s">
+        <v>18</v>
+      </c>
+      <c r="F22" s="9"/>
+      <c r="G22" s="9"/>
+      <c r="H22" s="9"/>
+    </row>
+    <row r="23" spans="2:8" s="12" customFormat="1" ht="58.5" x14ac:dyDescent="0.25">
+      <c r="B23" s="20" t="s">
+        <v>69</v>
+      </c>
+      <c r="C23" s="20" t="s">
+        <v>43</v>
+      </c>
+      <c r="D23" s="21" t="s">
+        <v>41</v>
+      </c>
+      <c r="E23" s="20" t="s">
+        <v>37</v>
+      </c>
+      <c r="F23" s="9"/>
+      <c r="G23" s="9"/>
+      <c r="H23" s="9"/>
+    </row>
+    <row r="24" spans="2:8" s="12" customFormat="1" ht="58.5" x14ac:dyDescent="0.25">
+      <c r="B24" s="20" t="s">
+        <v>70</v>
+      </c>
+      <c r="C24" s="21" t="s">
+        <v>44</v>
+      </c>
+      <c r="D24" s="21" t="s">
+        <v>41</v>
+      </c>
+      <c r="E24" s="20" t="s">
+        <v>23</v>
+      </c>
+      <c r="F24" s="9"/>
+      <c r="G24" s="9"/>
+      <c r="H24" s="9"/>
+    </row>
+    <row r="25" spans="2:8" s="12" customFormat="1" ht="19.5" x14ac:dyDescent="0.25">
+      <c r="B25" s="20"/>
+      <c r="C25" s="21"/>
+      <c r="D25" s="21"/>
+      <c r="E25" s="20"/>
+      <c r="F25" s="9"/>
+      <c r="G25" s="9"/>
+      <c r="H25" s="9"/>
+    </row>
+    <row r="26" spans="2:8" s="12" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B26" s="20" t="s">
+        <v>71</v>
+      </c>
+      <c r="C26" s="20" t="s">
+        <v>46</v>
+      </c>
+      <c r="D26" s="20" t="s">
+        <v>45</v>
+      </c>
+      <c r="E26" s="20" t="s">
+        <v>18</v>
+      </c>
+      <c r="F26" s="9"/>
+      <c r="G26" s="9"/>
+      <c r="H26" s="9"/>
+    </row>
+    <row r="27" spans="2:8" s="12" customFormat="1" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="B27" s="20" t="s">
+        <v>72</v>
+      </c>
+      <c r="C27" s="20" t="s">
+        <v>47</v>
+      </c>
+      <c r="D27" s="20" t="s">
+        <v>45</v>
+      </c>
+      <c r="E27" s="24" t="s">
+        <v>48</v>
+      </c>
+      <c r="F27" s="9"/>
+      <c r="G27" s="9"/>
+      <c r="H27" s="9"/>
+    </row>
+    <row r="28" spans="2:8" s="12" customFormat="1" ht="58.5" x14ac:dyDescent="0.25">
+      <c r="B28" s="20" t="s">
+        <v>73</v>
+      </c>
+      <c r="C28" s="21" t="s">
+        <v>49</v>
+      </c>
+      <c r="D28" s="20" t="s">
+        <v>45</v>
+      </c>
+      <c r="E28" s="20" t="s">
+        <v>50</v>
+      </c>
+      <c r="F28" s="9"/>
+      <c r="G28" s="9"/>
+      <c r="H28" s="9"/>
+    </row>
+    <row r="29" spans="2:8" s="12" customFormat="1" ht="19.5" x14ac:dyDescent="0.25">
+      <c r="B29" s="20" t="s">
+        <v>74</v>
+      </c>
+      <c r="C29" s="20" t="s">
+        <v>51</v>
+      </c>
+      <c r="D29" s="20" t="s">
+        <v>45</v>
+      </c>
+      <c r="E29" s="20" t="s">
+        <v>23</v>
+      </c>
+      <c r="F29" s="9"/>
+      <c r="G29" s="9"/>
+      <c r="H29" s="9"/>
+    </row>
+    <row r="30" spans="2:8" s="12" customFormat="1" ht="19.5" x14ac:dyDescent="0.25">
+      <c r="B30" s="24" t="s">
+        <v>75</v>
+      </c>
+      <c r="C30" s="21" t="s">
+        <v>52</v>
+      </c>
+      <c r="D30" s="20" t="s">
+        <v>45</v>
+      </c>
+      <c r="E30" s="20" t="s">
+        <v>23</v>
+      </c>
+      <c r="F30" s="9"/>
+      <c r="G30" s="9"/>
+      <c r="H30" s="9"/>
+    </row>
+    <row r="31" spans="2:8" s="12" customFormat="1" ht="19.5" x14ac:dyDescent="0.25">
+      <c r="B31" s="24" t="s">
+        <v>76</v>
+      </c>
+      <c r="C31" s="21" t="s">
+        <v>53</v>
+      </c>
+      <c r="D31" s="20" t="s">
+        <v>45</v>
+      </c>
+      <c r="E31" s="20" t="s">
+        <v>23</v>
+      </c>
+      <c r="F31" s="9"/>
+      <c r="G31" s="9"/>
+      <c r="H31" s="9"/>
+    </row>
+    <row r="32" spans="2:8" s="12" customFormat="1" ht="19.5" x14ac:dyDescent="0.25">
+      <c r="B32" s="24" t="s">
+        <v>77</v>
+      </c>
+      <c r="C32" s="21" t="s">
+        <v>54</v>
+      </c>
+      <c r="D32" s="20" t="s">
+        <v>45</v>
+      </c>
+      <c r="E32" s="20" t="s">
+        <v>37</v>
+      </c>
+      <c r="F32" s="9"/>
+      <c r="G32" s="9"/>
+      <c r="H32" s="9"/>
+    </row>
+    <row r="33" spans="2:8" s="12" customFormat="1" ht="19.5" x14ac:dyDescent="0.25">
+      <c r="B33" s="24" t="s">
+        <v>78</v>
+      </c>
+      <c r="C33" s="21" t="s">
+        <v>55</v>
+      </c>
+      <c r="D33" s="20" t="s">
+        <v>45</v>
+      </c>
+      <c r="E33" s="20" t="s">
+        <v>13</v>
+      </c>
+      <c r="F33" s="9"/>
+      <c r="G33" s="9"/>
+      <c r="H33" s="9"/>
+    </row>
+    <row r="34" spans="2:8" s="12" customFormat="1" ht="19.5" x14ac:dyDescent="0.25">
+      <c r="B34" s="24" t="s">
+        <v>79</v>
+      </c>
+      <c r="C34" s="21" t="s">
+        <v>56</v>
+      </c>
+      <c r="D34" s="20" t="s">
+        <v>45</v>
+      </c>
+      <c r="E34" s="20" t="s">
+        <v>13</v>
+      </c>
+      <c r="F34" s="9"/>
+      <c r="G34" s="9"/>
+      <c r="H34" s="9"/>
+    </row>
+    <row r="35" spans="2:8" s="12" customFormat="1" ht="19.5" x14ac:dyDescent="0.25">
+      <c r="B35" s="24" t="s">
+        <v>80</v>
+      </c>
+      <c r="C35" s="21" t="s">
+        <v>57</v>
+      </c>
+      <c r="D35" s="20" t="s">
+        <v>45</v>
+      </c>
+      <c r="E35" s="20" t="s">
+        <v>18</v>
+      </c>
+      <c r="F35" s="9"/>
+      <c r="G35" s="9"/>
+      <c r="H35" s="9"/>
+    </row>
+    <row r="36" spans="2:8" s="12" customFormat="1" ht="19.5" x14ac:dyDescent="0.25">
+      <c r="B36" s="20"/>
+      <c r="C36" s="21"/>
+      <c r="D36" s="20"/>
+      <c r="E36" s="20"/>
+      <c r="F36" s="9"/>
+      <c r="G36" s="9"/>
+      <c r="H36" s="9"/>
+    </row>
+    <row r="37" spans="2:8" s="12" customFormat="1" ht="58.5" x14ac:dyDescent="0.25">
+      <c r="B37" s="24" t="s">
+        <v>81</v>
+      </c>
+      <c r="C37" s="21" t="s">
+        <v>58</v>
+      </c>
+      <c r="D37" s="20" t="s">
+        <v>59</v>
+      </c>
+      <c r="E37" s="20" t="s">
+        <v>23</v>
+      </c>
+      <c r="F37" s="9"/>
+      <c r="G37" s="9"/>
+      <c r="H37" s="9"/>
+    </row>
+    <row r="38" spans="2:8" s="12" customFormat="1" ht="19.5" x14ac:dyDescent="0.25">
+      <c r="B38" s="24" t="s">
+        <v>82</v>
+      </c>
+      <c r="C38" s="21" t="s">
+        <v>60</v>
+      </c>
+      <c r="D38" s="20" t="s">
+        <v>59</v>
+      </c>
+      <c r="E38" s="20" t="s">
+        <v>13</v>
+      </c>
+      <c r="F38" s="9"/>
+      <c r="G38" s="9"/>
+      <c r="H38" s="9"/>
+    </row>
+    <row r="39" spans="2:8" s="12" customFormat="1" ht="19.5" x14ac:dyDescent="0.25">
+      <c r="B39" s="20"/>
+      <c r="C39" s="21"/>
+      <c r="D39" s="20"/>
+      <c r="E39" s="20"/>
+      <c r="F39" s="9"/>
+      <c r="G39" s="9"/>
+      <c r="H39" s="9"/>
+    </row>
+    <row r="40" spans="2:8" s="12" customFormat="1" ht="39" x14ac:dyDescent="0.25">
+      <c r="B40" s="24" t="s">
+        <v>83</v>
+      </c>
+      <c r="C40" s="21" t="s">
+        <v>61</v>
+      </c>
+      <c r="D40" s="21" t="s">
+        <v>62</v>
+      </c>
+      <c r="E40" s="20" t="s">
+        <v>18</v>
+      </c>
+      <c r="F40" s="9"/>
+      <c r="G40" s="9"/>
+      <c r="H40" s="9"/>
+    </row>
+    <row r="41" spans="2:8" s="12" customFormat="1" ht="19.5" x14ac:dyDescent="0.25">
+      <c r="B41" s="20"/>
+      <c r="C41" s="21"/>
+      <c r="D41" s="20"/>
+      <c r="E41" s="20"/>
+      <c r="F41" s="9"/>
+      <c r="G41" s="9"/>
+      <c r="H41" s="9"/>
+    </row>
+    <row r="42" spans="2:8" s="12" customFormat="1" ht="39" x14ac:dyDescent="0.25">
+      <c r="B42" s="24" t="s">
+        <v>84</v>
+      </c>
+      <c r="C42" s="21" t="s">
+        <v>63</v>
+      </c>
+      <c r="D42" s="21" t="s">
+        <v>65</v>
+      </c>
+      <c r="E42" s="20" t="s">
+        <v>64</v>
+      </c>
+      <c r="F42" s="9"/>
+      <c r="G42" s="9"/>
+      <c r="H42" s="9"/>
+    </row>
+    <row r="43" spans="2:8" s="12" customFormat="1" ht="19.5" x14ac:dyDescent="0.25">
+      <c r="B43" s="20"/>
+      <c r="C43" s="21"/>
+      <c r="D43" s="21"/>
+      <c r="E43" s="20"/>
+      <c r="F43" s="9"/>
+      <c r="G43" s="9"/>
+      <c r="H43" s="9"/>
+    </row>
+    <row r="44" spans="2:8" s="12" customFormat="1" ht="19.5" x14ac:dyDescent="0.25">
+      <c r="B44" s="20" t="s">
+        <v>94</v>
+      </c>
+      <c r="C44" s="21" t="s">
+        <v>87</v>
+      </c>
+      <c r="D44" s="21" t="s">
+        <v>85</v>
+      </c>
+      <c r="E44" s="20" t="s">
+        <v>88</v>
+      </c>
+      <c r="F44" s="9"/>
+      <c r="G44" s="9"/>
+      <c r="H44" s="9"/>
+    </row>
+    <row r="45" spans="2:8" s="12" customFormat="1" ht="19.5" x14ac:dyDescent="0.25">
+      <c r="B45" s="20" t="s">
+        <v>95</v>
+      </c>
+      <c r="C45" s="21" t="s">
+        <v>86</v>
+      </c>
+      <c r="D45" s="21" t="s">
+        <v>85</v>
+      </c>
+      <c r="E45" s="20" t="s">
+        <v>23</v>
+      </c>
+      <c r="F45" s="9"/>
+      <c r="G45" s="9"/>
+      <c r="H45" s="9"/>
+    </row>
+    <row r="46" spans="2:8" s="12" customFormat="1" ht="19.5" x14ac:dyDescent="0.25">
+      <c r="B46" s="20" t="s">
+        <v>96</v>
+      </c>
+      <c r="C46" s="21" t="s">
+        <v>89</v>
+      </c>
+      <c r="D46" s="21" t="s">
+        <v>85</v>
+      </c>
+      <c r="E46" s="20" t="s">
+        <v>90</v>
+      </c>
+      <c r="F46" s="9"/>
+      <c r="G46" s="9"/>
+      <c r="H46" s="9"/>
+    </row>
+    <row r="47" spans="2:8" s="12" customFormat="1" ht="19.5" x14ac:dyDescent="0.25">
+      <c r="B47" s="20"/>
+      <c r="C47" s="21"/>
+      <c r="D47" s="21"/>
+      <c r="E47" s="20"/>
+      <c r="F47" s="9"/>
+      <c r="G47" s="9"/>
+      <c r="H47" s="9"/>
+    </row>
+    <row r="48" spans="2:8" s="12" customFormat="1" ht="39" x14ac:dyDescent="0.25">
+      <c r="B48" s="20" t="s">
+        <v>97</v>
+      </c>
+      <c r="C48" s="21" t="s">
+        <v>92</v>
+      </c>
+      <c r="D48" s="21" t="s">
+        <v>91</v>
+      </c>
+      <c r="E48" s="20" t="s">
+        <v>93</v>
+      </c>
+      <c r="F48" s="9"/>
+      <c r="G48" s="9"/>
+      <c r="H48" s="9"/>
+    </row>
+    <row r="49" spans="2:8" s="12" customFormat="1" ht="39" x14ac:dyDescent="0.25">
+      <c r="B49" s="20" t="s">
+        <v>99</v>
+      </c>
+      <c r="C49" s="21" t="s">
+        <v>98</v>
+      </c>
+      <c r="D49" s="21" t="s">
+        <v>91</v>
+      </c>
+      <c r="E49" s="24" t="s">
+        <v>48</v>
+      </c>
+      <c r="F49" s="9"/>
+      <c r="G49" s="9"/>
+      <c r="H49" s="9"/>
+    </row>
+    <row r="50" spans="2:8" s="12" customFormat="1" ht="39" x14ac:dyDescent="0.25">
+      <c r="B50" s="20" t="s">
+        <v>100</v>
+      </c>
+      <c r="C50" s="21" t="s">
+        <v>102</v>
+      </c>
+      <c r="D50" s="21" t="s">
+        <v>91</v>
+      </c>
+      <c r="E50" s="24" t="s">
+        <v>101</v>
+      </c>
+      <c r="F50" s="9"/>
+      <c r="G50" s="9"/>
+      <c r="H50" s="9"/>
+    </row>
+    <row r="51" spans="2:8" s="12" customFormat="1" ht="39" x14ac:dyDescent="0.25">
+      <c r="B51" s="20" t="s">
+        <v>108</v>
+      </c>
+      <c r="C51" s="21" t="s">
+        <v>103</v>
+      </c>
+      <c r="D51" s="21" t="s">
+        <v>91</v>
+      </c>
+      <c r="E51" s="24" t="s">
+        <v>48</v>
+      </c>
+      <c r="F51" s="9"/>
+      <c r="G51" s="9"/>
+      <c r="H51" s="9"/>
+    </row>
+    <row r="52" spans="2:8" s="12" customFormat="1" ht="39" x14ac:dyDescent="0.25">
+      <c r="B52" s="20" t="s">
+        <v>109</v>
+      </c>
+      <c r="C52" s="21" t="s">
+        <v>104</v>
+      </c>
+      <c r="D52" s="21" t="s">
+        <v>91</v>
+      </c>
+      <c r="E52" s="24" t="s">
+        <v>93</v>
+      </c>
+      <c r="F52" s="9"/>
+      <c r="G52" s="9"/>
+      <c r="H52" s="9"/>
+    </row>
+    <row r="53" spans="2:8" s="12" customFormat="1" ht="39" x14ac:dyDescent="0.25">
+      <c r="B53" s="20" t="s">
+        <v>110</v>
+      </c>
+      <c r="C53" s="21" t="s">
+        <v>105</v>
+      </c>
+      <c r="D53" s="21" t="s">
+        <v>91</v>
+      </c>
+      <c r="E53" s="24" t="s">
+        <v>93</v>
+      </c>
+      <c r="F53" s="9"/>
+      <c r="G53" s="9"/>
+      <c r="H53" s="9"/>
+    </row>
+    <row r="54" spans="2:8" s="12" customFormat="1" ht="39" x14ac:dyDescent="0.25">
+      <c r="B54" s="20" t="s">
+        <v>111</v>
+      </c>
+      <c r="C54" s="21" t="s">
+        <v>106</v>
+      </c>
+      <c r="D54" s="21" t="s">
+        <v>91</v>
+      </c>
+      <c r="E54" s="24" t="s">
+        <v>101</v>
+      </c>
+      <c r="F54" s="9"/>
+      <c r="G54" s="9"/>
+      <c r="H54" s="9"/>
+    </row>
+    <row r="55" spans="2:8" s="12" customFormat="1" ht="58.5" x14ac:dyDescent="0.25">
+      <c r="B55" s="20" t="s">
+        <v>112</v>
+      </c>
+      <c r="C55" s="21" t="s">
+        <v>107</v>
+      </c>
+      <c r="D55" s="21" t="s">
+        <v>91</v>
+      </c>
+      <c r="E55" s="24" t="s">
+        <v>93</v>
+      </c>
+      <c r="F55" s="9"/>
+      <c r="G55" s="9"/>
+      <c r="H55" s="9"/>
+    </row>
+    <row r="56" spans="2:8" s="12" customFormat="1" ht="19.5" x14ac:dyDescent="0.25">
+      <c r="B56" s="20"/>
+      <c r="C56" s="21"/>
+      <c r="D56" s="21"/>
+      <c r="E56" s="24"/>
+      <c r="F56" s="9"/>
+      <c r="G56" s="9"/>
+      <c r="H56" s="9"/>
+    </row>
+    <row r="57" spans="2:8" s="12" customFormat="1" ht="39" x14ac:dyDescent="0.25">
+      <c r="B57" s="20" t="s">
+        <v>118</v>
+      </c>
+      <c r="C57" s="21" t="s">
+        <v>113</v>
+      </c>
+      <c r="D57" s="21" t="s">
+        <v>116</v>
+      </c>
+      <c r="E57" s="24" t="s">
+        <v>34</v>
+      </c>
+      <c r="F57" s="9"/>
+      <c r="G57" s="9"/>
+      <c r="H57" s="9"/>
+    </row>
+    <row r="58" spans="2:8" s="12" customFormat="1" ht="39" x14ac:dyDescent="0.25">
+      <c r="B58" s="20" t="s">
+        <v>119</v>
+      </c>
+      <c r="C58" s="21" t="s">
+        <v>114</v>
+      </c>
+      <c r="D58" s="21" t="s">
+        <v>116</v>
+      </c>
+      <c r="E58" s="24" t="s">
+        <v>115</v>
+      </c>
+      <c r="F58" s="9"/>
+      <c r="G58" s="9"/>
+      <c r="H58" s="9"/>
+    </row>
+    <row r="59" spans="2:8" s="12" customFormat="1" ht="39" x14ac:dyDescent="0.25">
+      <c r="B59" s="20" t="s">
+        <v>120</v>
+      </c>
+      <c r="C59" s="21" t="s">
+        <v>117</v>
+      </c>
+      <c r="D59" s="21" t="s">
+        <v>116</v>
+      </c>
+      <c r="E59" s="24" t="s">
+        <v>34</v>
+      </c>
+      <c r="F59" s="9"/>
+      <c r="G59" s="9"/>
+      <c r="H59" s="9"/>
+    </row>
+    <row r="61" spans="2:8" ht="18" x14ac:dyDescent="0.25">
+      <c r="B61" s="8"/>
+      <c r="C61" s="8"/>
+      <c r="D61" s="10"/>
+      <c r="E61" s="8"/>
+      <c r="F61" s="8"/>
+      <c r="G61" s="8"/>
+      <c r="H61" s="8"/>
+    </row>
+    <row r="63" spans="2:8" ht="18" x14ac:dyDescent="0.25">
+      <c r="B63" s="8"/>
+      <c r="C63" s="8"/>
+      <c r="D63" s="8"/>
+      <c r="E63" s="8"/>
+      <c r="F63" s="8"/>
+      <c r="G63" s="8"/>
+      <c r="H63" s="8"/>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="B1:H1"/>
+    <mergeCell ref="B2:H2"/>
+    <mergeCell ref="B3:H3"/>
+  </mergeCells>
+  <printOptions horizontalCentered="1" verticalCentered="1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" scale="80" orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>